<commit_message>
Added code for multiple cell values from Excel using data provider
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\srini\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD3161F4-9652-480B-A8E0-CAC36795D163}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59B29F28-C470-4EEB-B11A-3ED752009575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Products" sheetId="1" r:id="rId1"/>
     <sheet name="Cart" sheetId="2" r:id="rId2"/>
-    <sheet name="DB_CustomerInfo" sheetId="3" r:id="rId3"/>
+    <sheet name="MultipleProducts" sheetId="4" r:id="rId3"/>
+    <sheet name="DB_CustomerInfo" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="22">
   <si>
     <t>TC_ID</t>
   </si>
@@ -84,6 +85,15 @@
   </si>
   <si>
     <t>Tpt</t>
+  </si>
+  <si>
+    <t>Sauce Labs Bolt T-Shirt</t>
+  </si>
+  <si>
+    <t>Sauce Labs Bike Light</t>
+  </si>
+  <si>
+    <t>Sauce Labs Fleece Jacket</t>
   </si>
 </sst>
 </file>
@@ -113,7 +123,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -121,14 +131,31 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -493,6 +520,44 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A11335B5-2DC4-4031-AEDF-290E141FB5F3}">
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="31.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB7DF562-5E6F-43F4-B155-D9F9AF008341}">
   <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>